<commit_message>
Translate TSSR template to English
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CRWK7dKrVv6aAx3STJqBmT
</commit_message>
<xml_diff>
--- a/tssr-lite/TSSR_lite.xlsx
+++ b/tssr-lite/TSSR_lite.xlsx
@@ -515,30 +515,30 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TSSR – uproszczony raport z wizji lokalnej</t>
+          <t>TSSR – simplified site survey report</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Do uzupełnienia:</t>
+          <t>Status:</t>
         </is>
       </c>
       <c r="E1" s="2">
-        <f>IF(((B4="")+(B5="")+(B6="")+(B7="")+(B8="")+(B9="")+(B10="")+(B11="")+(B16="")+(B17="")+(B20="")+(B105="")+(B106="")+(B107="")+(B108="")+(B109="")+(B110=""))=0,"✔ komplet",((B4="")+(B5="")+(B6="")+(B7="")+(B8="")+(B9="")+(B10="")+(B11="")+(B16="")+(B17="")+(B20="")+(B105="")+(B106="")+(B107="")+(B108="")+(B109="")+(B110=""))&amp;" pól obowiązkowych brakuje")</f>
+        <f>IF(((B4="")+(B5="")+(B6="")+(B7="")+(B8="")+(B9="")+(B10="")+(B11="")+(B16="")+(B17="")+(B20="")+(B105="")+(B106="")+(B107="")+(B108="")+(B109="")+(B110=""))=0,"✔ complete",((B4="")+(B5="")+(B6="")+(B7="")+(B8="")+(B9="")+(B10="")+(B11="")+(B16="")+(B17="")+(B20="")+(B105="")+(B106="")+(B107="")+(B108="")+(B109="")+(B110=""))&amp;" mandatory fields missing")</f>
         <v/>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Żółte = do wypełnienia, szare = automat, białe = opcjonalne. Nic więcej nie trzeba.</t>
+          <t>Yellow = fill in, grey = automatic, white = optional.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>1. LOKALIZACJA</t>
+          <t>1. SITE</t>
         </is>
       </c>
       <c r="B3" s="5" t="n"/>
@@ -549,7 +549,7 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Kod site'u</t>
+          <t>Site code</t>
         </is>
       </c>
       <c r="B4" s="7" t="n"/>
@@ -560,7 +560,7 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Nazwa site'u</t>
+          <t>Site name</t>
         </is>
       </c>
       <c r="B5" s="7" t="n"/>
@@ -571,7 +571,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Adres</t>
+          <t>Address</t>
         </is>
       </c>
       <c r="B6" s="7" t="n"/>
@@ -582,7 +582,7 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Współrzędne GPS (lat, lon)</t>
+          <t>GPS coordinates (lat, lon)</t>
         </is>
       </c>
       <c r="B7" s="7" t="n"/>
@@ -593,7 +593,7 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Klient / projekt</t>
+          <t>Client / project</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -608,7 +608,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Typ lokalizacji</t>
+          <t>Site type</t>
         </is>
       </c>
       <c r="B9" s="7" t="n"/>
@@ -619,7 +619,7 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Data wizji</t>
+          <t>Survey date</t>
         </is>
       </c>
       <c r="B10" s="7" t="n"/>
@@ -630,7 +630,7 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Kto robił wizję (imię, firma, tel.)</t>
+          <t>Surveyor (name, company, phone)</t>
         </is>
       </c>
       <c r="B11" s="7" t="n"/>
@@ -641,7 +641,7 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Kontakt do dostępu na site (imię, tel.)</t>
+          <t>Site access contact (name, phone)</t>
         </is>
       </c>
       <c r="B12" s="9" t="n"/>
@@ -652,7 +652,7 @@
     <row r="13" ht="95" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Uwagi do dostępu (klucze, godziny, ptaki/pszczoły itp.)</t>
+          <t>Access notes (keys, hours, bird nests / bee hives etc.)</t>
         </is>
       </c>
       <c r="B13" s="9" t="n"/>
@@ -663,7 +663,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>2. ROZWIĄZANIE (najważniejsze)</t>
+          <t>2. SOLUTION (most important)</t>
         </is>
       </c>
       <c r="B15" s="5" t="n"/>
@@ -674,7 +674,7 @@
     <row r="16" ht="95" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Opis planowanego rozwiązania</t>
+          <t>Description of planned solution</t>
         </is>
       </c>
       <c r="B16" s="7" t="n"/>
@@ -685,7 +685,7 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Typ swapu</t>
+          <t>Swap type</t>
         </is>
       </c>
       <c r="B17" s="7" t="n"/>
@@ -696,7 +696,7 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Szafa indoor</t>
+          <t>Indoor cabinet</t>
         </is>
       </c>
       <c r="B18" s="9" t="n"/>
@@ -707,7 +707,7 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Szafa outdoor</t>
+          <t>Outdoor cabinet</t>
         </is>
       </c>
       <c r="B19" s="9" t="n"/>
@@ -718,7 +718,7 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Środki specjalne (dźwig / podnośnik)</t>
+          <t>Special means (crane / cherry picker)</t>
         </is>
       </c>
       <c r="B20" s="7" t="n"/>
@@ -729,7 +729,7 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Czas prac (swap)</t>
+          <t>Swap duration</t>
         </is>
       </c>
       <c r="B21" s="9" t="n"/>
@@ -740,7 +740,7 @@
     <row r="22" ht="95" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>Prace cywilne / stalowe potrzebne? (opisz)</t>
+          <t>Civil / steel works needed? (describe)</t>
         </is>
       </c>
       <c r="B22" s="9" t="n"/>
@@ -751,7 +751,7 @@
     <row r="23" ht="95" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>Konfiguracja docelowa (sektory, pasma, BB, anteny – skrót)</t>
+          <t>Target configuration (sectors, bands, BB, antennas – summary)</t>
         </is>
       </c>
       <c r="B23" s="9" t="n"/>
@@ -762,7 +762,7 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>3. SPRZĘT NOKIA DO ZAMÓWIENIA  (wybierz z listy, wpisz ilość)</t>
+          <t>3. NOKIA HW TO ORDER  (pick from list, enter quantity)</t>
         </is>
       </c>
       <c r="B25" s="5" t="n"/>
@@ -773,23 +773,23 @@
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>Wybierz pozycję z listy</t>
+          <t>Pick item from list</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>Nr części (auto)</t>
+          <t>Part no. (auto)</t>
         </is>
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>Ilość</t>
+          <t>Qty</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr"/>
       <c r="E26" s="10" t="inlineStr">
         <is>
-          <t>Uwagi</t>
+          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1096,7 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>4. MATERIAŁY INSTALACYJNE (kable, jumpery, uchwyty)</t>
+          <t>4. INSTALLATION MATERIALS (cables, jumpers, clamps)</t>
         </is>
       </c>
       <c r="B58" s="5" t="n"/>
@@ -1107,23 +1107,23 @@
     <row r="59">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>Wybierz pozycję z listy</t>
+          <t>Pick item from list</t>
         </is>
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>Kod (auto)</t>
+          <t>Code (auto)</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
         <is>
-          <t>Ilość</t>
+          <t>Qty</t>
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr"/>
       <c r="E59" s="10" t="inlineStr">
         <is>
-          <t>Uwagi</t>
+          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -1380,7 +1380,7 @@
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>5. DO DEMONTAŻU (anteny, RRU, BTS – wpisz typ i ilość)</t>
+          <t>5. TO BE REMOVED (antennas, RRU, BTS – enter type and qty)</t>
         </is>
       </c>
       <c r="B86" s="5" t="n"/>
@@ -1391,23 +1391,23 @@
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>Co demontujemy</t>
+          <t>Item to remove</t>
         </is>
       </c>
       <c r="B87" s="10" t="inlineStr">
         <is>
-          <t>Lokalizacja / sektor</t>
+          <t>Location / sector</t>
         </is>
       </c>
       <c r="C87" s="10" t="inlineStr">
         <is>
-          <t>Ilość</t>
+          <t>Qty</t>
         </is>
       </c>
       <c r="D87" s="10" t="inlineStr"/>
       <c r="E87" s="10" t="inlineStr">
         <is>
-          <t>Uwagi</t>
+          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1519,7 @@
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>6. BEZPIECZEŃSTWO I ZASILANIE (krótko)</t>
+          <t>6. SAFETY AND POWER (brief)</t>
         </is>
       </c>
       <c r="B104" s="5" t="n"/>
@@ -1530,7 +1530,7 @@
     <row r="105">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>Czy można bezpiecznie wykonać prace?</t>
+          <t>Can the work be carried out safely?</t>
         </is>
       </c>
       <c r="B105" s="7" t="n"/>
@@ -1541,7 +1541,7 @@
     <row r="106">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>Czy potrzebny dźwig / podnośnik?</t>
+          <t>Is a crane / cherry picker needed?</t>
         </is>
       </c>
       <c r="B106" s="7" t="n"/>
@@ -1552,7 +1552,7 @@
     <row r="107">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>Czy potrzebne rusztowanie?</t>
+          <t>Is scaffolding needed?</t>
         </is>
       </c>
       <c r="B107" s="7" t="n"/>
@@ -1563,7 +1563,7 @@
     <row r="108">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>Podejrzenie azbestu / materiałów niebezpiecznych?</t>
+          <t>Suspected asbestos / hazardous materials?</t>
         </is>
       </c>
       <c r="B108" s="7" t="n"/>
@@ -1574,7 +1574,7 @@
     <row r="109">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>Czy trzeba zwiększyć zasilanie AC / dołożyć bezpieczniki?</t>
+          <t>AC power increase / new breakers needed?</t>
         </is>
       </c>
       <c r="B109" s="7" t="n"/>
@@ -1585,7 +1585,7 @@
     <row r="110">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>Czy potrzebny nowy prostownik / DCDU?</t>
+          <t>New rectifier / DCDU needed?</t>
         </is>
       </c>
       <c r="B110" s="7" t="n"/>
@@ -1596,7 +1596,7 @@
     <row r="111" ht="95" customHeight="1">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>Zasilanie – co jest teraz i czego brakuje</t>
+          <t>Power – current state and what is missing</t>
         </is>
       </c>
       <c r="B111" s="9" t="n"/>
@@ -1607,7 +1607,7 @@
     <row r="112" ht="95" customHeight="1">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>Znalezione usterki / zagrożenia / inne uwagi</t>
+          <t>Deficiencies / hazards / other remarks found</t>
         </is>
       </c>
       <c r="B112" s="9" t="n"/>
@@ -1618,7 +1618,7 @@
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>7. ZDJĘCIA (osobno, w folderze / na dysku – nie wklejamy tutaj)</t>
+          <t>7. PHOTOS (separate, in a folder – do not paste here)</t>
         </is>
       </c>
       <c r="B114" s="5" t="n"/>
@@ -1629,21 +1629,21 @@
     <row r="115" ht="18" customHeight="1">
       <c r="A115" s="14" t="inlineStr">
         <is>
-          <t>Nazewnictwo plików:  KODSITE_01_widok-ogolny.jpg, KODSITE_02_dojazd.jpg …</t>
+          <t>File naming:  SITECODE_01_general-view.jpg, SITECODE_02_access-road.jpg …</t>
         </is>
       </c>
     </row>
     <row r="116" ht="32" customHeight="1">
       <c r="A116" s="14" t="inlineStr">
         <is>
-          <t>Minimum: widok na site i z site'u, dojazd/wejście, szafa/pomieszczenie, zasilanie (AC i DC), maszt/dach przy antenach, każdy sektor (antena + RRU), trasy kablowe, miejsca na nowy sprzęt.</t>
+          <t>Minimum: view of the site and from the site, access road/entrance, cabinet/room, power (AC and DC), tower/roof at the antennas, each sector (antenna + RRU), cable routes, locations for new equipment.</t>
         </is>
       </c>
     </row>
     <row r="117" ht="18" customHeight="1">
       <c r="A117" s="14" t="inlineStr">
         <is>
-          <t>Link do folderu ze zdjęciami:</t>
+          <t>Link to photo folder:</t>
         </is>
       </c>
     </row>
@@ -1793,54 +1793,54 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>TAK/NIE</t>
+          <t>YES/NO</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Typ swapu</t>
+          <t>Swap type</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>Pomieszczenie / szafa indoor</t>
+          <t>Indoor cabinet / rack</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Szafa outdoor</t>
+          <t>Outdoor cabinet</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Środki specjalne</t>
+          <t>Special means</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>Czas</t>
+          <t>Duration</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>Typ lokalizacji</t>
+          <t>Site type</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t>Sprzęt Nokia (PN – opis)</t>
+          <t>Nokia HW (PN – description)</t>
         </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>Materiały instalacyjne (kod – opis)</t>
+          <t>Installation materials (code – description)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TAK</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1860,12 +1860,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Brak</t>
+          <t>None</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1/2 dnia</t>
+          <t>1/2 day</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1887,7 +1887,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>NIE</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1907,12 +1907,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Cherry Picker do 45 m</t>
+          <t>Cherry Picker up to 45 m</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1 dzień</t>
+          <t>1 day</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1934,7 +1934,7 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>Inny (opisz)</t>
+          <t>Other (describe)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1949,12 +1949,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Cherry Picker powyżej 45 m</t>
+          <t>Cherry Picker over 45 m</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2 dni</t>
+          <t>2 days</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1981,17 +1981,17 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Brak</t>
+          <t>None</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Dźwig powyżej 45 t</t>
+          <t>Crane over 45 t</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Więcej</t>
+          <t>More</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2013,12 +2013,12 @@
     <row r="6">
       <c r="C6" t="inlineStr">
         <is>
-          <t>Brak</t>
+          <t>None</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Inny</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">

</xml_diff>